<commit_message>
Title: Fix OpenCV import error in questionnaire extractor
Key features implemented:
- Added explicit OpenCV import at the beginning of detect_checkboxes function to resolve ModuleNotFoundError
- Updated test assets including new test image (test_page.png) and updated test output (test_output.xlsx) for validation
- Modified .gitignore handling to properly manage Excel binary files

The changes address the critical runtime error while maintaining compatibility with existing functionality and improving test coverage.
</commit_message>
<xml_diff>
--- a/test_output.xlsx
+++ b/test_output.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>Vraag (Question)</t>
   </si>
@@ -64,85 +64,31 @@
     <t>Hoe wil jij dit nieuws zien?</t>
   </si>
   <si>
-    <t>Waar ging dat nieuws over?</t>
-  </si>
-  <si>
-    <t>Ging dit nieuws over jouw buurt, stad of regio?</t>
+    <t>M v x -OO</t>
+  </si>
+  <si>
+    <t>3s S)</t>
+  </si>
+  <si>
+    <t>Gedeeld, met iemand besproken? Ben je ergens naartoe gegaan? ae</t>
   </si>
   <si>
     <t>Wat voor bericht was het?</t>
   </si>
   <si>
-    <t>Hoe ben je bij dit nieuws gekomen?</t>
-  </si>
-  <si>
-    <t>Gedeeld, met iemand besproken?</t>
-  </si>
-  <si>
-    <t>Ben je ergens naartoe gegaan?</t>
-  </si>
-  <si>
-    <t>Verder gezocht naar meer nieuws over zelfde onderwerp?</t>
-  </si>
-  <si>
-    <t>Of juist niets gedaan, waarom?</t>
-  </si>
-  <si>
-    <t>Waarom wel niet:</t>
-  </si>
-  <si>
-    <t>Interessant, Relevant, Boeiend, Toegankelijk?</t>
-  </si>
-  <si>
-    <t>Gaat over jou / jongeren?</t>
-  </si>
-  <si>
-    <t>Had invloed op je dagelijks leven?</t>
-  </si>
-  <si>
-    <t>Kon je er wat mee? raakte jou persoonlijk?</t>
-  </si>
-  <si>
-    <t>voelde je beter geïnformeerd?</t>
-  </si>
-  <si>
-    <t>Het veranderde iets aan wat je deed of dacht?</t>
-  </si>
-  <si>
-    <t>Dagdeel, redactiesessie, 50 euro vergoeding. noteer e-mail</t>
-  </si>
-  <si>
-    <t>Platform</t>
-  </si>
-  <si>
-    <t>Vorm</t>
-  </si>
-  <si>
-    <t>M Vv Xx 7b LIU</t>
-  </si>
-  <si>
-    <t>° ee "</t>
-  </si>
-  <si>
-    <t>11 [_] Laatste nieuws [_]Sport [ | Tech &amp; Innovatie [ | 112-nieuws [| Klimaat [ | Reizen &amp; Avontuur [| Health &amp; Mindset [_]Activisme &amp; Impact [ | Veiligheid &amp; Criminaliteit [| Geld &amp; Carriére [ | Entertainment [_ ]Cultuur [ | Studie &amp; Ontwikkeling [ | Lifestyle; (Inhoud) over moet gaan? Kun je een top 3 geven?</t>
-  </si>
-  <si>
-    <t>[_ ] Politiek &amp; Maatschappij</t>
-  </si>
-  <si>
-    <t>betekent e Lifestyle e faat zien hoe ik er zelf mee te maken heb ¢ mij iets nieuws leert e¢ betrouwbaar voelt e kort en duidelijk is</t>
-  </si>
-  <si>
-    <t>diepgang heeft ¢ Veiligheid &amp; Criminaliteit e verschillende kanten van een verhaal e Entertainment laat zien e Studie &amp; Ontwikkeling ¢ ook laat zien wat wél werkt en welke ° Politiek &amp; Maatschappij kansen er zijn ¢ Sport e niet alleen negatief is, maar ook e 112-nieuws positieve dingen laat zien e Reizen &amp; Avontuur e boeiend en makkelijk te begrijpen is © Activisme &amp; Impact</t>
-  </si>
-  <si>
-    <t>vervolgonderzoek?</t>
-  </si>
-  <si>
-    <t>H il jij dit ni on?</t>
-  </si>
-  <si>
-    <t>Platform Vorm</t>
+    <t>° en “</t>
+  </si>
+  <si>
+    <t>11 [_] Laatste nieuws [Sport (Tech &amp; Innovatie ([]112-nieuws []Klimaat [_]Reizen &amp; Avontuur [Health &amp; Mindset [_JActivisme &amp; Impact [_]veiligheid &amp; Criminaliteit_ [Geld &amp; Carriére [JEntertainment (_Jeultuur [_JStudie &amp; Ontwikkeling [Lifestyle</t>
+  </si>
+  <si>
+    <t>Ht il jij dit ni san?</t>
+  </si>
+  <si>
+    <t>Of juist niets gedaan, waarom? vervolgonderzoek? 8 oe Dagdeel, redactiesessie, 50 euro vergoeding. noteer e-mail</t>
+  </si>
+  <si>
+    <t>loe wil jij dit nieuws zien? Had invioed op je dagelijks leven? Platform Vorm voelde je beter geinformeerd?</t>
   </si>
 </sst>
 </file>
@@ -500,7 +446,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B33"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -521,13 +467,16 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
         <v>4</v>
       </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
@@ -543,18 +492,24 @@
       <c r="A7" t="s">
         <v>7</v>
       </c>
+      <c r="B7" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
         <v>8</v>
       </c>
+      <c r="B8" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
         <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -567,7 +522,7 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -580,122 +535,23 @@
         <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>37</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
         <v>14</v>
       </c>
+      <c r="B14" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="16" spans="1:2">
-      <c r="A16" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2">
-      <c r="A17" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2">
-      <c r="A18" t="s">
-        <v>18</v>
-      </c>
-      <c r="B18" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2">
-      <c r="A19" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2">
-      <c r="A20" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2">
-      <c r="A21" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2">
-      <c r="A22" t="s">
-        <v>22</v>
-      </c>
-      <c r="B22" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2">
-      <c r="A23" t="s">
-        <v>23</v>
-      </c>
-      <c r="B23" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2">
-      <c r="A24" t="s">
+      <c r="B15" t="s">
         <v>24</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2">
-      <c r="A25" t="s">
-        <v>25</v>
-      </c>
-      <c r="B25" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2">
-      <c r="A26" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2">
-      <c r="A27" t="s">
-        <v>27</v>
-      </c>
-      <c r="B27" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2">
-      <c r="A28" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2">
-      <c r="A29" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2">
-      <c r="A30" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2">
-      <c r="A31" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2">
-      <c r="A32" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1">
-      <c r="A33" t="s">
-        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>